<commit_message>
Ext ADC data streaming OK
</commit_message>
<xml_diff>
--- a/readme_imgs/Book1.xlsx
+++ b/readme_imgs/Book1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jougasaki_\Desktop\ecg_stm_proj\readme_imgs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PHONK\Desktop\ecg_stm\readme_imgs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D24E221-832A-44D1-B47E-B43546840366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6020DD0-480C-48BB-A106-510E80955EF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{6C4AAC5D-AEFA-471A-9DCC-ACAC6EDD2760}"/>
+    <workbookView xWindow="-21720" yWindow="-9480" windowWidth="21840" windowHeight="38040" xr2:uid="{6C4AAC5D-AEFA-471A-9DCC-ACAC6EDD2760}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -537,7 +537,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="27">
   <si>
     <t>Address</t>
   </si>
@@ -615,6 +615,9 @@
   </si>
   <si>
     <t>FILTER3</t>
+  </si>
+  <si>
+    <t>Остальные регистры - кастомные коэфы для фильтров и какая-то хрень для CRC как я понял, похер на них</t>
   </si>
 </sst>
 </file>
@@ -827,58 +830,58 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -896,10 +899,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1222,467 +1221,472 @@
   <dimension ref="A1:R14"/>
   <sheetFormatPr defaultColWidth="4" defaultRowHeight="22.5" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="4" style="2"/>
+    <col min="1" max="16384" width="4" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="8" t="s">
+      <c r="A1" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="9"/>
-      <c r="F1" s="10">
+      <c r="E1" s="18"/>
+      <c r="F1" s="5">
         <v>7</v>
       </c>
-      <c r="G1" s="10">
+      <c r="G1" s="5">
         <v>6</v>
       </c>
-      <c r="H1" s="10">
+      <c r="H1" s="5">
         <v>5</v>
       </c>
-      <c r="I1" s="10">
+      <c r="I1" s="5">
         <v>4</v>
       </c>
-      <c r="J1" s="10">
+      <c r="J1" s="5">
         <v>3</v>
       </c>
-      <c r="K1" s="10">
+      <c r="K1" s="5">
         <v>2</v>
       </c>
-      <c r="L1" s="10">
+      <c r="L1" s="5">
         <v>1</v>
       </c>
-      <c r="M1" s="11">
-        <v>0</v>
-      </c>
-      <c r="N1" s="4" t="s">
+      <c r="M1" s="6">
+        <v>0</v>
+      </c>
+      <c r="N1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="7"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="15"/>
     </row>
     <row r="2" spans="1:18" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="13">
-        <v>0</v>
-      </c>
-      <c r="G2" s="5">
+      <c r="E2" s="13"/>
+      <c r="F2" s="2">
+        <v>0</v>
+      </c>
+      <c r="G2" s="3">
         <v>1</v>
       </c>
-      <c r="H2" s="5">
-        <v>0</v>
-      </c>
-      <c r="I2" s="5">
+      <c r="H2" s="3">
+        <v>0</v>
+      </c>
+      <c r="I2" s="3">
         <v>1</v>
       </c>
-      <c r="J2" s="5">
+      <c r="J2" s="3">
         <v>1</v>
       </c>
-      <c r="K2" s="5">
-        <v>0</v>
-      </c>
-      <c r="L2" s="5">
-        <v>0</v>
-      </c>
-      <c r="M2" s="6">
-        <v>0</v>
-      </c>
-      <c r="N2" s="12" t="s">
+      <c r="K2" s="3">
+        <v>0</v>
+      </c>
+      <c r="L2" s="3">
+        <v>0</v>
+      </c>
+      <c r="M2" s="4">
+        <v>0</v>
+      </c>
+      <c r="N2" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="O2" s="12"/>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
+      <c r="O2" s="16"/>
+      <c r="P2" s="16"/>
+      <c r="Q2" s="16"/>
+      <c r="R2" s="16"/>
     </row>
     <row r="3" spans="1:18" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1" t="s">
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="1"/>
-      <c r="F3" s="2" t="s">
+      <c r="E3" s="13"/>
+      <c r="F3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L3" s="17">
-        <v>0</v>
-      </c>
-      <c r="M3" s="17">
-        <v>0</v>
-      </c>
-      <c r="N3" s="1" t="s">
+      <c r="L3" s="10">
+        <v>0</v>
+      </c>
+      <c r="M3" s="10">
+        <v>0</v>
+      </c>
+      <c r="N3" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="O3" s="1"/>
-      <c r="P3" s="1"/>
-      <c r="Q3" s="1"/>
-      <c r="R3" s="1"/>
+      <c r="O3" s="13"/>
+      <c r="P3" s="13"/>
+      <c r="Q3" s="13"/>
+      <c r="R3" s="13"/>
     </row>
     <row r="4" spans="1:18" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1" t="s">
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="1"/>
-      <c r="F4" s="15">
-        <v>0</v>
-      </c>
-      <c r="G4" s="15">
-        <v>0</v>
-      </c>
-      <c r="H4" s="15">
+      <c r="E4" s="13"/>
+      <c r="F4" s="8">
+        <v>0</v>
+      </c>
+      <c r="G4" s="8">
+        <v>0</v>
+      </c>
+      <c r="H4" s="8">
         <v>1</v>
       </c>
-      <c r="I4" s="15">
-        <v>0</v>
-      </c>
-      <c r="J4" s="16" t="s">
+      <c r="I4" s="8">
+        <v>0</v>
+      </c>
+      <c r="J4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="K4" s="16" t="s">
+      <c r="K4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="L4" s="16" t="s">
+      <c r="L4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="M4" s="16" t="s">
+      <c r="M4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="N4" s="1" t="s">
+      <c r="N4" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="O4" s="1"/>
-      <c r="P4" s="1"/>
-      <c r="Q4" s="1"/>
-      <c r="R4" s="1"/>
+      <c r="O4" s="13"/>
+      <c r="P4" s="13"/>
+      <c r="Q4" s="13"/>
+      <c r="R4" s="13"/>
     </row>
     <row r="5" spans="1:18" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1" t="s">
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="1"/>
-      <c r="F5" s="2" t="s">
+      <c r="E5" s="13"/>
+      <c r="F5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="14">
+      <c r="H5" s="7">
         <v>1</v>
       </c>
-      <c r="I5" s="6">
-        <v>0</v>
-      </c>
-      <c r="J5" s="13">
-        <v>0</v>
-      </c>
-      <c r="K5" s="6">
+      <c r="I5" s="4">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2">
+        <v>0</v>
+      </c>
+      <c r="K5" s="4">
         <v>1</v>
       </c>
-      <c r="L5" s="15">
-        <v>0</v>
-      </c>
-      <c r="M5" s="15">
-        <v>0</v>
-      </c>
-      <c r="N5" s="1" t="s">
+      <c r="L5" s="8">
+        <v>0</v>
+      </c>
+      <c r="M5" s="8">
+        <v>0</v>
+      </c>
+      <c r="N5" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="O5" s="1"/>
-      <c r="P5" s="1"/>
-      <c r="Q5" s="1"/>
-      <c r="R5" s="1"/>
+      <c r="O5" s="13"/>
+      <c r="P5" s="13"/>
+      <c r="Q5" s="13"/>
+      <c r="R5" s="13"/>
     </row>
     <row r="6" spans="1:18" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1" t="s">
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="1"/>
-      <c r="F6" s="15">
-        <v>0</v>
-      </c>
-      <c r="G6" s="13">
-        <v>0</v>
-      </c>
-      <c r="H6" s="6">
-        <v>0</v>
-      </c>
-      <c r="I6" s="18" t="s">
+      <c r="E6" s="13"/>
+      <c r="F6" s="8">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4">
+        <v>0</v>
+      </c>
+      <c r="I6" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="J6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K6" s="19">
-        <v>0</v>
-      </c>
-      <c r="L6" s="19">
-        <v>0</v>
-      </c>
-      <c r="M6" s="19">
-        <v>0</v>
-      </c>
-      <c r="N6" s="1" t="s">
+      <c r="K6" s="12">
+        <v>0</v>
+      </c>
+      <c r="L6" s="12">
+        <v>0</v>
+      </c>
+      <c r="M6" s="12">
+        <v>0</v>
+      </c>
+      <c r="N6" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="O6" s="1"/>
-      <c r="P6" s="1"/>
-      <c r="Q6" s="1"/>
-      <c r="R6" s="1"/>
+      <c r="O6" s="13"/>
+      <c r="P6" s="13"/>
+      <c r="Q6" s="13"/>
+      <c r="R6" s="13"/>
     </row>
     <row r="7" spans="1:18" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1" t="s">
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="1"/>
-      <c r="F7" s="13">
-        <v>0</v>
-      </c>
-      <c r="G7" s="5">
-        <v>0</v>
-      </c>
-      <c r="H7" s="6">
-        <v>0</v>
-      </c>
-      <c r="I7" s="13">
-        <v>0</v>
-      </c>
-      <c r="J7" s="5">
-        <v>0</v>
-      </c>
-      <c r="K7" s="5">
-        <v>0</v>
-      </c>
-      <c r="L7" s="5">
-        <v>0</v>
-      </c>
-      <c r="M7" s="6">
+      <c r="E7" s="13"/>
+      <c r="F7" s="2">
+        <v>0</v>
+      </c>
+      <c r="G7" s="3">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4">
+        <v>0</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0</v>
+      </c>
+      <c r="J7" s="3">
+        <v>0</v>
+      </c>
+      <c r="K7" s="3">
+        <v>0</v>
+      </c>
+      <c r="L7" s="3">
+        <v>0</v>
+      </c>
+      <c r="M7" s="4">
         <v>1</v>
       </c>
-      <c r="N7" s="1" t="s">
+      <c r="N7" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
-      <c r="Q7" s="1"/>
-      <c r="R7" s="1"/>
+      <c r="O7" s="13"/>
+      <c r="P7" s="13"/>
+      <c r="Q7" s="13"/>
+      <c r="R7" s="13"/>
     </row>
     <row r="8" spans="1:18" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1" t="s">
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="1"/>
-      <c r="F8" s="2" t="s">
+      <c r="E8" s="13"/>
+      <c r="F8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G8" s="13">
-        <v>0</v>
-      </c>
-      <c r="H8" s="5">
-        <v>0</v>
-      </c>
-      <c r="I8" s="6">
-        <v>0</v>
-      </c>
-      <c r="J8" s="15">
-        <v>0</v>
-      </c>
-      <c r="K8" s="15">
-        <v>0</v>
-      </c>
-      <c r="L8" s="15">
-        <v>0</v>
-      </c>
-      <c r="M8" s="15">
+      <c r="G8" s="2">
+        <v>0</v>
+      </c>
+      <c r="H8" s="3">
+        <v>0</v>
+      </c>
+      <c r="I8" s="4">
+        <v>0</v>
+      </c>
+      <c r="J8" s="8">
+        <v>0</v>
+      </c>
+      <c r="K8" s="8">
+        <v>0</v>
+      </c>
+      <c r="L8" s="8">
+        <v>0</v>
+      </c>
+      <c r="M8" s="8">
         <v>1</v>
       </c>
-      <c r="N8" s="1" t="s">
+      <c r="N8" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="O8" s="1"/>
-      <c r="P8" s="1"/>
-      <c r="Q8" s="1"/>
-      <c r="R8" s="1"/>
+      <c r="O8" s="13"/>
+      <c r="P8" s="13"/>
+      <c r="Q8" s="13"/>
+      <c r="R8" s="13"/>
     </row>
     <row r="9" spans="1:18" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="2" t="s">
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="J9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="K9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L9" s="13">
-        <v>0</v>
-      </c>
-      <c r="M9" s="6">
-        <v>0</v>
-      </c>
-      <c r="N9" s="1" t="s">
+      <c r="L9" s="2">
+        <v>0</v>
+      </c>
+      <c r="M9" s="4">
+        <v>0</v>
+      </c>
+      <c r="N9" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="O9" s="1"/>
-      <c r="P9" s="1"/>
-      <c r="Q9" s="1"/>
-      <c r="R9" s="1"/>
+      <c r="O9" s="13"/>
+      <c r="P9" s="13"/>
+      <c r="Q9" s="13"/>
+      <c r="R9" s="13"/>
     </row>
     <row r="10" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="N10" s="1"/>
-      <c r="O10" s="1"/>
-      <c r="P10" s="1"/>
-      <c r="Q10" s="1"/>
-      <c r="R10" s="1"/>
+      <c r="A10" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
+      <c r="J10" s="13"/>
+      <c r="K10" s="13"/>
+      <c r="L10" s="13"/>
+      <c r="M10" s="13"/>
+      <c r="N10" s="13"/>
+      <c r="O10" s="13"/>
+      <c r="P10" s="13"/>
+      <c r="Q10" s="13"/>
+      <c r="R10" s="13"/>
     </row>
     <row r="11" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="N11" s="1"/>
-      <c r="O11" s="1"/>
-      <c r="P11" s="1"/>
-      <c r="Q11" s="1"/>
-      <c r="R11" s="1"/>
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="13"/>
+      <c r="K11" s="13"/>
+      <c r="L11" s="13"/>
+      <c r="M11" s="13"/>
+      <c r="N11" s="13"/>
+      <c r="O11" s="13"/>
+      <c r="P11" s="13"/>
+      <c r="Q11" s="13"/>
+      <c r="R11" s="13"/>
     </row>
     <row r="12" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
-      <c r="P12" s="1"/>
-      <c r="Q12" s="1"/>
-      <c r="R12" s="1"/>
+      <c r="A12" s="13"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="N12" s="13"/>
+      <c r="O12" s="13"/>
+      <c r="P12" s="13"/>
+      <c r="Q12" s="13"/>
+      <c r="R12" s="13"/>
     </row>
     <row r="13" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="1"/>
-      <c r="Q13" s="1"/>
-      <c r="R13" s="1"/>
+      <c r="A13" s="13"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="N13" s="13"/>
+      <c r="O13" s="13"/>
+      <c r="P13" s="13"/>
+      <c r="Q13" s="13"/>
+      <c r="R13" s="13"/>
     </row>
     <row r="14" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
-      <c r="P14" s="1"/>
-      <c r="Q14" s="1"/>
-      <c r="R14" s="1"/>
+      <c r="A14" s="13"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="N14" s="13"/>
+      <c r="O14" s="13"/>
+      <c r="P14" s="13"/>
+      <c r="Q14" s="13"/>
+      <c r="R14" s="13"/>
     </row>
   </sheetData>
-  <mergeCells count="42">
-    <mergeCell ref="N11:R11"/>
-    <mergeCell ref="N12:R12"/>
-    <mergeCell ref="N13:R13"/>
-    <mergeCell ref="N14:R14"/>
-    <mergeCell ref="N5:R5"/>
-    <mergeCell ref="N6:R6"/>
-    <mergeCell ref="N7:R7"/>
-    <mergeCell ref="N8:R8"/>
-    <mergeCell ref="N9:R9"/>
-    <mergeCell ref="N10:R10"/>
-    <mergeCell ref="N1:R1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="N2:R2"/>
-    <mergeCell ref="N3:R3"/>
-    <mergeCell ref="N4:R4"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
+  <mergeCells count="37">
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A10:R11"/>
     <mergeCell ref="D14:E14"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A14:C14"/>
@@ -1697,14 +1701,22 @@
     <mergeCell ref="A7:C7"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="N1:R1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="N2:R2"/>
+    <mergeCell ref="N3:R3"/>
+    <mergeCell ref="N4:R4"/>
+    <mergeCell ref="N12:R12"/>
+    <mergeCell ref="N13:R13"/>
+    <mergeCell ref="N14:R14"/>
+    <mergeCell ref="N5:R5"/>
+    <mergeCell ref="N6:R6"/>
+    <mergeCell ref="N7:R7"/>
+    <mergeCell ref="N8:R8"/>
+    <mergeCell ref="N9:R9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>